<commit_message>
config wszystkich baz danych
</commit_message>
<xml_diff>
--- a/DistributedDbs.xlsx
+++ b/DistributedDbs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Coding\Studia\Praca-Magisterka-Distributed-Sql\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{685E17B1-0EF4-433B-BD19-F2651C7FF700}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46679EA2-DC36-4990-85F7-BD723BCD377B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="57480" yWindow="7980" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="68">
   <si>
     <t>Nazwa</t>
   </si>
@@ -245,6 +245,9 @@
   </si>
   <si>
     <t>uruchomiony (tylko mysql)</t>
+  </si>
+  <si>
+    <t>Docker (local)</t>
   </si>
 </sst>
 </file>
@@ -942,6 +945,9 @@
       <c r="C16" t="s">
         <v>5</v>
       </c>
+      <c r="D16" t="s">
+        <v>67</v>
+      </c>
       <c r="E16" s="7" t="s">
         <v>60</v>
       </c>

</xml_diff>